<commit_message>
contacts added for ward 1
</commit_message>
<xml_diff>
--- a/New Microsoft Excel Worksheet.xlsx
+++ b/New Microsoft Excel Worksheet.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\082_083\ward1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D324B80-E6C5-40BB-8BA0-568CC1F90A4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -32,6 +33,88 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>User</author>
+  </authors>
+  <commentList>
+    <comment ref="D4" authorId="0" shapeId="0" xr:uid="{AD28CD2A-6F95-4BA7-BF55-9966A86999EB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+bhadra</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{9336CFC1-3459-4BF8-B3A8-5B5478745621}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Ashwin</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{8713AFB4-3DF0-432A-8F9E-0D0B99DA63F9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Kartik</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
   <si>
@@ -128,8 +211,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,6 +238,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -205,12 +301,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -221,11 +311,17 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -505,92 +601,92 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AB19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.109375" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="4.33203125" customWidth="1"/>
-    <col min="4" max="5" width="8.88671875" style="7"/>
-    <col min="6" max="6" width="6.21875" customWidth="1"/>
-    <col min="7" max="7" width="8.88671875" style="11"/>
-    <col min="11" max="11" width="8.88671875" style="11"/>
-    <col min="13" max="13" width="7.21875" customWidth="1"/>
-    <col min="14" max="14" width="5.109375" customWidth="1"/>
-    <col min="15" max="15" width="8.5546875" style="7" customWidth="1"/>
-    <col min="16" max="16" width="8" style="11" customWidth="1"/>
-    <col min="17" max="17" width="6.88671875" customWidth="1"/>
-    <col min="18" max="18" width="7.6640625" customWidth="1"/>
-    <col min="20" max="20" width="8.88671875" customWidth="1"/>
-    <col min="21" max="21" width="14.44140625" customWidth="1"/>
-    <col min="22" max="22" width="8.88671875" style="7"/>
-    <col min="24" max="24" width="8.88671875" style="14"/>
-    <col min="27" max="27" width="8.88671875" customWidth="1"/>
+    <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.140625" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="4.28515625" customWidth="1"/>
+    <col min="4" max="5" width="8.85546875" style="5"/>
+    <col min="6" max="6" width="6.28515625" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" style="9"/>
+    <col min="11" max="11" width="8.85546875" style="9"/>
+    <col min="13" max="13" width="7.28515625" customWidth="1"/>
+    <col min="14" max="14" width="5.140625" customWidth="1"/>
+    <col min="15" max="15" width="8.5703125" style="5" customWidth="1"/>
+    <col min="16" max="16" width="8" style="9" customWidth="1"/>
+    <col min="17" max="17" width="6.85546875" customWidth="1"/>
+    <col min="18" max="18" width="7.7109375" customWidth="1"/>
+    <col min="20" max="20" width="8.85546875" customWidth="1"/>
+    <col min="21" max="21" width="14.42578125" customWidth="1"/>
+    <col min="22" max="22" width="8.85546875" style="5"/>
+    <col min="24" max="24" width="8.85546875" style="11"/>
+    <col min="27" max="27" width="8.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:28" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4" t="s">
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="12" t="s">
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="5" t="s">
+      <c r="R1" s="13"/>
+      <c r="S1" s="13"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13"/>
+      <c r="V1" s="13"/>
+      <c r="W1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="X1" s="12" t="s">
+      <c r="X1" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="Y1" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="Z1" s="5" t="s">
+      <c r="Z1" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="AA1" s="5" t="s">
+      <c r="AA1" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AB1" s="12" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
+    <row r="2" spans="1:28" s="6" customFormat="1" ht="71.25" x14ac:dyDescent="0.25">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
@@ -600,7 +696,7 @@
       <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H2" s="3" t="s">
@@ -612,7 +708,7 @@
       <c r="J2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="7" t="s">
         <v>6</v>
       </c>
       <c r="L2" s="3" t="s">
@@ -627,7 +723,7 @@
       <c r="O2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="12"/>
+      <c r="P2" s="14"/>
       <c r="Q2" s="3" t="s">
         <v>14</v>
       </c>
@@ -646,26 +742,26 @@
       <c r="V2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="W2" s="5"/>
-      <c r="X2" s="12"/>
-      <c r="Y2" s="5"/>
-      <c r="Z2" s="5"/>
-      <c r="AA2" s="5"/>
-      <c r="AB2" s="5"/>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="W2" s="12"/>
+      <c r="X2" s="14"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="12"/>
+      <c r="AB2" s="12"/>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="6">
+      <c r="D3" s="4">
         <v>32902</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="4">
         <f>ROUNDUP(D3/30,0)*4</f>
         <v>4388</v>
       </c>
       <c r="F3" s="2"/>
-      <c r="G3" s="10">
+      <c r="G3" s="8">
         <f>SUM(D3:F3)</f>
         <v>37290</v>
       </c>
@@ -680,7 +776,7 @@
         <f>6%*G3</f>
         <v>2237.4</v>
       </c>
-      <c r="K3" s="10">
+      <c r="K3" s="8">
         <f>SUM(G3:J3)</f>
         <v>43656.4</v>
       </c>
@@ -691,11 +787,11 @@
         <v>0</v>
       </c>
       <c r="N3" s="2"/>
-      <c r="O3" s="6">
+      <c r="O3" s="4">
         <f>SUM(L3:M3)</f>
         <v>2000</v>
       </c>
-      <c r="P3" s="10">
+      <c r="P3" s="8">
         <f>K3+O3</f>
         <v>45656.4</v>
       </c>
@@ -714,7 +810,7 @@
         <f>J3*2</f>
         <v>4474.8</v>
       </c>
-      <c r="V3" s="6">
+      <c r="V3" s="4">
         <f>SUM(Q3:U3)</f>
         <v>17732.8</v>
       </c>
@@ -722,7 +818,7 @@
         <f>X3+U3</f>
         <v>32398.400000000001</v>
       </c>
-      <c r="X3" s="13">
+      <c r="X3" s="10">
         <f>P3-V3</f>
         <v>27923.600000000002</v>
       </c>
@@ -737,19 +833,19 @@
       <c r="AA3" s="2"/>
       <c r="AB3" s="2"/>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="6">
+      <c r="D4" s="4">
         <v>34730</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="4">
         <f>ROUNDUP(D4/30,0)*4</f>
         <v>4632</v>
       </c>
       <c r="F4" s="2"/>
-      <c r="G4" s="10">
+      <c r="G4" s="8">
         <f>SUM(D4:F4)</f>
         <v>39362</v>
       </c>
@@ -764,7 +860,7 @@
         <f>6%*G4</f>
         <v>2361.7199999999998</v>
       </c>
-      <c r="K4" s="10">
+      <c r="K4" s="8">
         <f>SUM(G4:J4)</f>
         <v>46059.92</v>
       </c>
@@ -777,11 +873,11 @@
         <v>39362</v>
       </c>
       <c r="N4" s="2"/>
-      <c r="O4" s="6">
+      <c r="O4" s="4">
         <f>SUM(L4:M4)</f>
         <v>44362</v>
       </c>
-      <c r="P4" s="10">
+      <c r="P4" s="8">
         <f>K4+O4</f>
         <v>90421.92</v>
       </c>
@@ -800,7 +896,7 @@
         <f>J4*2</f>
         <v>4723.4399999999996</v>
       </c>
-      <c r="V4" s="6">
+      <c r="V4" s="4">
         <f>SUM(Q4:U4)</f>
         <v>18395.84</v>
       </c>
@@ -808,7 +904,7 @@
         <f>X4+U4</f>
         <v>76749.52</v>
       </c>
-      <c r="X4" s="13">
+      <c r="X4" s="10">
         <f>P4-V4</f>
         <v>72026.080000000002</v>
       </c>
@@ -823,19 +919,19 @@
       <c r="AA4" s="2"/>
       <c r="AB4" s="2"/>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>34730</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="4">
         <f>ROUNDUP(D5/30,0)*4</f>
         <v>4632</v>
       </c>
       <c r="F5" s="2"/>
-      <c r="G5" s="10">
+      <c r="G5" s="8">
         <f>SUM(D5:F5)</f>
         <v>39362</v>
       </c>
@@ -850,7 +946,7 @@
         <f>6%*G5</f>
         <v>2361.7199999999998</v>
       </c>
-      <c r="K5" s="10">
+      <c r="K5" s="8">
         <f>SUM(G5:J5)</f>
         <v>46059.92</v>
       </c>
@@ -862,16 +958,16 @@
         <v>0</v>
       </c>
       <c r="N5" s="2"/>
-      <c r="O5" s="6">
+      <c r="O5" s="4">
         <f>SUM(L5:M5)</f>
         <v>5000</v>
       </c>
-      <c r="P5" s="10">
+      <c r="P5" s="8">
         <f>K5+O5</f>
         <v>51059.92</v>
       </c>
       <c r="Q5" s="2">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="R5" s="2">
         <f>H5*2</f>
@@ -885,17 +981,17 @@
         <f>J5*2</f>
         <v>4723.4399999999996</v>
       </c>
-      <c r="V5" s="6">
+      <c r="V5" s="4">
         <f>SUM(Q5:U5)</f>
-        <v>18396.84</v>
+        <v>18395.84</v>
       </c>
       <c r="W5" s="2">
         <f>X5+U5</f>
-        <v>37386.519999999997</v>
-      </c>
-      <c r="X5" s="13">
+        <v>37387.519999999997</v>
+      </c>
+      <c r="X5" s="10">
         <f>P5-V5</f>
-        <v>32663.079999999998</v>
+        <v>32664.079999999998</v>
       </c>
       <c r="Y5" s="2">
         <f>IF(X5*13&gt;600000,1%*X5,0)</f>
@@ -903,40 +999,41 @@
       </c>
       <c r="Z5" s="2">
         <f>X5-Y5</f>
-        <v>32663.079999999998</v>
+        <v>32664.079999999998</v>
       </c>
       <c r="AA5" s="2"/>
       <c r="AB5" s="2"/>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="6">
-        <v>43689</v>
-      </c>
-      <c r="E6" s="6">
-        <v>0</v>
+      <c r="D6" s="4">
+        <v>34730</v>
+      </c>
+      <c r="E6" s="4">
+        <f>ROUNDUP(D6/30,0)*4</f>
+        <v>4632</v>
       </c>
       <c r="F6" s="2"/>
-      <c r="G6" s="10">
+      <c r="G6" s="8">
         <f>SUM(D6:F6)</f>
-        <v>43689</v>
+        <v>39362</v>
       </c>
       <c r="H6" s="2">
         <f>10%*G6</f>
-        <v>4368.9000000000005</v>
+        <v>3936.2000000000003</v>
       </c>
       <c r="I6" s="2">
         <v>400</v>
       </c>
       <c r="J6" s="2">
         <f>6%*G6</f>
-        <v>2621.3399999999997</v>
-      </c>
-      <c r="K6" s="10">
+        <v>2361.7199999999998</v>
+      </c>
+      <c r="K6" s="8">
         <f>SUM(G6:J6)</f>
-        <v>51079.24</v>
+        <v>46059.92</v>
       </c>
       <c r="L6" s="2">
         <f>2000+3000</f>
@@ -946,40 +1043,40 @@
         <v>0</v>
       </c>
       <c r="N6" s="2"/>
-      <c r="O6" s="6">
+      <c r="O6" s="4">
         <f>SUM(L6:M6)</f>
         <v>5000</v>
       </c>
-      <c r="P6" s="10">
+      <c r="P6" s="8">
         <f>K6+O6</f>
-        <v>56079.24</v>
+        <v>51059.92</v>
       </c>
       <c r="Q6" s="2">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="R6" s="2">
         <f>H6*2</f>
-        <v>8737.8000000000011</v>
+        <v>7872.4000000000005</v>
       </c>
       <c r="S6" s="2">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="T6" s="2"/>
       <c r="U6" s="2">
         <f>J6*2</f>
-        <v>5242.6799999999994</v>
-      </c>
-      <c r="V6" s="6">
+        <v>4723.4399999999996</v>
+      </c>
+      <c r="V6" s="4">
         <f>SUM(Q6:U6)</f>
-        <v>15781.48</v>
+        <v>18395.84</v>
       </c>
       <c r="W6" s="2">
         <f>X6+U6</f>
-        <v>45540.439999999995</v>
-      </c>
-      <c r="X6" s="13">
+        <v>37387.519999999997</v>
+      </c>
+      <c r="X6" s="10">
         <f>P6-V6</f>
-        <v>40297.759999999995</v>
+        <v>32664.079999999998</v>
       </c>
       <c r="Y6" s="2">
         <f>IF(X6*13&gt;600000,1%*X6,0)</f>
@@ -987,310 +1084,454 @@
       </c>
       <c r="Z6" s="2">
         <f>X6-Y6</f>
-        <v>40297.759999999995</v>
+        <v>32664.079999999998</v>
       </c>
       <c r="AA6" s="2"/>
       <c r="AB6" s="2"/>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
       <c r="F7" s="2"/>
-      <c r="G7" s="10"/>
+      <c r="G7" s="8"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
-      <c r="K7" s="10"/>
+      <c r="K7" s="8"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
-      <c r="O7" s="6"/>
-      <c r="P7" s="10"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="8"/>
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
-      <c r="V7" s="6"/>
+      <c r="V7" s="4"/>
       <c r="W7" s="2"/>
-      <c r="X7" s="13"/>
+      <c r="X7" s="10"/>
       <c r="Y7" s="2"/>
       <c r="Z7" s="2"/>
       <c r="AA7" s="2"/>
       <c r="AB7" s="2"/>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
       <c r="F8" s="2"/>
-      <c r="G8" s="10"/>
+      <c r="G8" s="8"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="10"/>
+      <c r="K8" s="8"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="10"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="8"/>
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
       <c r="T8" s="2"/>
       <c r="U8" s="2"/>
-      <c r="V8" s="6"/>
+      <c r="V8" s="4"/>
       <c r="W8" s="2"/>
-      <c r="X8" s="13"/>
+      <c r="X8" s="10"/>
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
       <c r="AA8" s="2"/>
       <c r="AB8" s="2"/>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
+      <c r="D9" s="4">
+        <v>43689</v>
+      </c>
+      <c r="E9" s="4">
+        <v>0</v>
+      </c>
       <c r="F9" s="2"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
+      <c r="G9" s="8">
+        <f>SUM(D9:F9)</f>
+        <v>43689</v>
+      </c>
+      <c r="H9" s="2">
+        <f>10%*G9</f>
+        <v>4368.9000000000005</v>
+      </c>
+      <c r="I9" s="2">
+        <v>400</v>
+      </c>
+      <c r="J9" s="2">
+        <f>6%*G9</f>
+        <v>2621.3399999999997</v>
+      </c>
+      <c r="K9" s="8">
+        <f>SUM(G9:J9)</f>
+        <v>51079.24</v>
+      </c>
+      <c r="L9" s="2">
+        <f>2000+3000</f>
+        <v>5000</v>
+      </c>
+      <c r="M9" s="2">
+        <v>0</v>
+      </c>
       <c r="N9" s="2"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="2"/>
+      <c r="O9" s="4">
+        <f>SUM(L9:M9)</f>
+        <v>5000</v>
+      </c>
+      <c r="P9" s="8">
+        <f>K9+O9</f>
+        <v>56079.24</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>801</v>
+      </c>
+      <c r="R9" s="2">
+        <f>H9*2</f>
+        <v>8737.8000000000011</v>
+      </c>
+      <c r="S9" s="2">
+        <v>1000</v>
+      </c>
       <c r="T9" s="2"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="2"/>
-      <c r="X9" s="13"/>
-      <c r="Y9" s="2"/>
-      <c r="Z9" s="2"/>
+      <c r="U9" s="2">
+        <f>J9*2</f>
+        <v>5242.6799999999994</v>
+      </c>
+      <c r="V9" s="4">
+        <f>SUM(Q9:U9)</f>
+        <v>15781.48</v>
+      </c>
+      <c r="W9" s="2">
+        <f>X9+U9</f>
+        <v>45540.439999999995</v>
+      </c>
+      <c r="X9" s="10">
+        <f>P9-V9</f>
+        <v>40297.759999999995</v>
+      </c>
+      <c r="Y9" s="2">
+        <f>IF(X9*13&gt;600000,1%*X9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z9" s="2">
+        <f>X9-Y9</f>
+        <v>40297.759999999995</v>
+      </c>
       <c r="AA9" s="2"/>
       <c r="AB9" s="2"/>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
       <c r="F10" s="2"/>
-      <c r="G10" s="10"/>
+      <c r="G10" s="8"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="10"/>
+      <c r="K10" s="8"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="10"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="8"/>
       <c r="Q10" s="2"/>
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
       <c r="T10" s="2"/>
       <c r="U10" s="2"/>
-      <c r="V10" s="6"/>
+      <c r="V10" s="4"/>
       <c r="W10" s="2"/>
-      <c r="X10" s="13"/>
+      <c r="X10" s="10"/>
       <c r="Y10" s="2"/>
       <c r="Z10" s="2"/>
       <c r="AA10" s="2"/>
       <c r="AB10" s="2"/>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
       <c r="F11" s="2"/>
-      <c r="G11" s="10"/>
+      <c r="G11" s="8"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
-      <c r="K11" s="10"/>
+      <c r="K11" s="8"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="10"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="8"/>
       <c r="Q11" s="2"/>
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
-      <c r="V11" s="6"/>
+      <c r="V11" s="4"/>
       <c r="W11" s="2"/>
-      <c r="X11" s="13"/>
+      <c r="X11" s="10"/>
       <c r="Y11" s="2"/>
       <c r="Z11" s="2"/>
       <c r="AA11" s="2"/>
       <c r="AB11" s="2"/>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
       <c r="F12" s="2"/>
-      <c r="G12" s="10"/>
+      <c r="G12" s="8"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
-      <c r="K12" s="10"/>
+      <c r="K12" s="8"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="10"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="8"/>
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
       <c r="T12" s="2"/>
       <c r="U12" s="2"/>
-      <c r="V12" s="6"/>
+      <c r="V12" s="4"/>
       <c r="W12" s="2"/>
-      <c r="X12" s="13"/>
+      <c r="X12" s="10"/>
       <c r="Y12" s="2"/>
       <c r="Z12" s="2"/>
       <c r="AA12" s="2"/>
       <c r="AB12" s="2"/>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
       <c r="F13" s="2"/>
-      <c r="G13" s="10"/>
+      <c r="G13" s="8"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
-      <c r="K13" s="10"/>
+      <c r="K13" s="8"/>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="10"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="8"/>
       <c r="Q13" s="2"/>
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
-      <c r="V13" s="6"/>
+      <c r="V13" s="4"/>
       <c r="W13" s="2"/>
-      <c r="X13" s="13"/>
+      <c r="X13" s="10"/>
       <c r="Y13" s="2"/>
       <c r="Z13" s="2"/>
       <c r="AA13" s="2"/>
       <c r="AB13" s="2"/>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="10"/>
+      <c r="G14" s="8"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
-      <c r="K14" s="10"/>
+      <c r="K14" s="8"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
-      <c r="O14" s="6"/>
-      <c r="P14" s="10"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="8"/>
       <c r="Q14" s="2"/>
       <c r="R14" s="2"/>
       <c r="S14" s="2"/>
       <c r="T14" s="2"/>
       <c r="U14" s="2"/>
-      <c r="V14" s="6"/>
+      <c r="V14" s="4"/>
       <c r="W14" s="2"/>
-      <c r="X14" s="13"/>
+      <c r="X14" s="10"/>
       <c r="Y14" s="2"/>
       <c r="Z14" s="2"/>
       <c r="AA14" s="2"/>
       <c r="AB14" s="2"/>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
       <c r="F15" s="2"/>
-      <c r="G15" s="10"/>
+      <c r="G15" s="8"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
-      <c r="K15" s="10"/>
+      <c r="K15" s="8"/>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
-      <c r="O15" s="6"/>
-      <c r="P15" s="10"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="8"/>
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
       <c r="T15" s="2"/>
       <c r="U15" s="2"/>
-      <c r="V15" s="6"/>
+      <c r="V15" s="4"/>
       <c r="W15" s="2"/>
-      <c r="X15" s="13"/>
+      <c r="X15" s="10"/>
       <c r="Y15" s="2"/>
       <c r="Z15" s="2"/>
       <c r="AA15" s="2"/>
       <c r="AB15" s="2"/>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
       <c r="F16" s="2"/>
-      <c r="G16" s="10"/>
+      <c r="G16" s="8"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="10"/>
+      <c r="K16" s="8"/>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
-      <c r="O16" s="6"/>
-      <c r="P16" s="10"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="8"/>
       <c r="Q16" s="2"/>
       <c r="R16" s="2"/>
       <c r="S16" s="2"/>
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
-      <c r="V16" s="6"/>
+      <c r="V16" s="4"/>
       <c r="W16" s="2"/>
-      <c r="X16" s="13"/>
+      <c r="X16" s="10"/>
       <c r="Y16" s="2"/>
       <c r="Z16" s="2"/>
       <c r="AA16" s="2"/>
       <c r="AB16" s="2"/>
+    </row>
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2"/>
+      <c r="S17" s="2"/>
+      <c r="T17" s="2"/>
+      <c r="U17" s="2"/>
+      <c r="V17" s="4"/>
+      <c r="W17" s="2"/>
+      <c r="X17" s="10"/>
+      <c r="Y17" s="2"/>
+      <c r="Z17" s="2"/>
+      <c r="AA17" s="2"/>
+      <c r="AB17" s="2"/>
+    </row>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+      <c r="T18" s="2"/>
+      <c r="U18" s="2"/>
+      <c r="V18" s="4"/>
+      <c r="W18" s="2"/>
+      <c r="X18" s="10"/>
+      <c r="Y18" s="2"/>
+      <c r="Z18" s="2"/>
+      <c r="AA18" s="2"/>
+      <c r="AB18" s="2"/>
+    </row>
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="8"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
+      <c r="S19" s="2"/>
+      <c r="T19" s="2"/>
+      <c r="U19" s="2"/>
+      <c r="V19" s="4"/>
+      <c r="W19" s="2"/>
+      <c r="X19" s="10"/>
+      <c r="Y19" s="2"/>
+      <c r="Z19" s="2"/>
+      <c r="AA19" s="2"/>
+      <c r="AB19" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -1311,5 +1552,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
little change in salary sheet
</commit_message>
<xml_diff>
--- a/New Microsoft Excel Worksheet.xlsx
+++ b/New Microsoft Excel Worksheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D324B80-E6C5-40BB-8BA0-568CC1F90A4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA314E9E-2DE7-4550-8C33-A289610C30DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -108,6 +108,30 @@
           </rPr>
           <t xml:space="preserve">
 Kartik</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D7" authorId="0" shapeId="0" xr:uid="{B599E665-7579-4A84-B571-B267676937E2}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Mangsir</t>
         </r>
       </text>
     </comment>
@@ -1093,29 +1117,84 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
+      <c r="D7" s="4">
+        <v>34730</v>
+      </c>
+      <c r="E7" s="4">
+        <f>ROUNDUP(D7/30,0)*4</f>
+        <v>4632</v>
+      </c>
       <c r="F7" s="2"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
+      <c r="G7" s="8">
+        <f>SUM(D7:F7)</f>
+        <v>39362</v>
+      </c>
+      <c r="H7" s="2">
+        <f>10%*G7</f>
+        <v>3936.2000000000003</v>
+      </c>
+      <c r="I7" s="2">
+        <v>400</v>
+      </c>
+      <c r="J7" s="2">
+        <f>6%*G7</f>
+        <v>2361.7199999999998</v>
+      </c>
+      <c r="K7" s="8">
+        <f>SUM(G7:J7)</f>
+        <v>46059.92</v>
+      </c>
+      <c r="L7" s="2">
+        <f>2000+3000</f>
+        <v>5000</v>
+      </c>
+      <c r="M7" s="2">
+        <v>0</v>
+      </c>
       <c r="N7" s="2"/>
-      <c r="O7" s="4"/>
-      <c r="P7" s="8"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
+      <c r="O7" s="4">
+        <f>SUM(L7:M7)</f>
+        <v>5000</v>
+      </c>
+      <c r="P7" s="8">
+        <f>K7+O7</f>
+        <v>51059.92</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>800</v>
+      </c>
+      <c r="R7" s="2">
+        <f>H7*2</f>
+        <v>7872.4000000000005</v>
+      </c>
+      <c r="S7" s="2">
+        <v>5000</v>
+      </c>
       <c r="T7" s="2"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="4"/>
-      <c r="W7" s="2"/>
-      <c r="X7" s="10"/>
-      <c r="Y7" s="2"/>
-      <c r="Z7" s="2"/>
+      <c r="U7" s="2">
+        <f>J7*2</f>
+        <v>4723.4399999999996</v>
+      </c>
+      <c r="V7" s="4">
+        <f>SUM(Q7:U7)</f>
+        <v>18395.84</v>
+      </c>
+      <c r="W7" s="2">
+        <f>X7+U7</f>
+        <v>37387.519999999997</v>
+      </c>
+      <c r="X7" s="10">
+        <f>P7-V7</f>
+        <v>32664.079999999998</v>
+      </c>
+      <c r="Y7" s="2">
+        <f>IF(X7*13&gt;600000,1%*X7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z7" s="2">
+        <f>X7-Y7</f>
+        <v>32664.079999999998</v>
+      </c>
       <c r="AA7" s="2"/>
       <c r="AB7" s="2"/>
     </row>

</xml_diff>

<commit_message>
nabir sir msg of estimate of nepaltol khanal tol nepaldanda khanepaani and krishi upaj too
</commit_message>
<xml_diff>
--- a/New Microsoft Excel Worksheet.xlsx
+++ b/New Microsoft Excel Worksheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA314E9E-2DE7-4550-8C33-A289610C30DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F82F1D3E-A415-450B-B437-48686E68F5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -135,6 +135,72 @@
         </r>
       </text>
     </comment>
+    <comment ref="D8" authorId="0" shapeId="0" xr:uid="{87073B8F-9072-4EF6-B208-947AACA7D7EC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t>User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">
+poush</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D9" authorId="0" shapeId="0" xr:uid="{5E7E19E1-C15B-4922-ACAF-F55EACE46A00}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t>User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">
+Magh</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D10" authorId="0" shapeId="0" xr:uid="{DFCBDEA9-2C22-4E5E-9B42-6533BB080AF6}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t>User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">
+falgun</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -236,7 +302,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -275,6 +341,17 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
     </font>
   </fonts>
   <fills count="3">
@@ -626,7 +703,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB19"/>
+  <dimension ref="A1:AB22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
@@ -1202,29 +1279,84 @@
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
+      <c r="D8" s="4">
+        <v>34730</v>
+      </c>
+      <c r="E8" s="4">
+        <f t="shared" ref="E8:E10" si="0">ROUNDUP(D8/30,0)*4</f>
+        <v>4632</v>
+      </c>
       <c r="F8" s="2"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
+      <c r="G8" s="8">
+        <f t="shared" ref="G8:G10" si="1">SUM(D8:F8)</f>
+        <v>39362</v>
+      </c>
+      <c r="H8" s="2">
+        <f t="shared" ref="H8:H10" si="2">10%*G8</f>
+        <v>3936.2000000000003</v>
+      </c>
+      <c r="I8" s="2">
+        <v>400</v>
+      </c>
+      <c r="J8" s="2">
+        <f t="shared" ref="J8:J10" si="3">6%*G8</f>
+        <v>2361.7199999999998</v>
+      </c>
+      <c r="K8" s="8">
+        <f t="shared" ref="K8:K10" si="4">SUM(G8:J8)</f>
+        <v>46059.92</v>
+      </c>
+      <c r="L8" s="2">
+        <f t="shared" ref="L8:L10" si="5">2000+3000</f>
+        <v>5000</v>
+      </c>
+      <c r="M8" s="2">
+        <v>0</v>
+      </c>
       <c r="N8" s="2"/>
-      <c r="O8" s="4"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
+      <c r="O8" s="4">
+        <f t="shared" ref="O8:O10" si="6">SUM(L8:M8)</f>
+        <v>5000</v>
+      </c>
+      <c r="P8" s="8">
+        <f t="shared" ref="P8:P10" si="7">K8+O8</f>
+        <v>51059.92</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>800</v>
+      </c>
+      <c r="R8" s="2">
+        <f t="shared" ref="R8:R10" si="8">H8*2</f>
+        <v>7872.4000000000005</v>
+      </c>
+      <c r="S8" s="2">
+        <v>5000</v>
+      </c>
       <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="4"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="10"/>
-      <c r="Y8" s="2"/>
-      <c r="Z8" s="2"/>
+      <c r="U8" s="2">
+        <f t="shared" ref="U8:U10" si="9">J8*2</f>
+        <v>4723.4399999999996</v>
+      </c>
+      <c r="V8" s="4">
+        <f t="shared" ref="V8:V10" si="10">SUM(Q8:U8)</f>
+        <v>18395.84</v>
+      </c>
+      <c r="W8" s="2">
+        <f t="shared" ref="W8:W10" si="11">X8+U8</f>
+        <v>37387.519999999997</v>
+      </c>
+      <c r="X8" s="10">
+        <f t="shared" ref="X8:X10" si="12">P8-V8</f>
+        <v>32664.079999999998</v>
+      </c>
+      <c r="Y8" s="2">
+        <f t="shared" ref="Y8:Y10" si="13">IF(X8*13&gt;600000,1%*X8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z8" s="2">
+        <f t="shared" ref="Z8:Z10" si="14">X8-Y8</f>
+        <v>32664.079999999998</v>
+      </c>
       <c r="AA8" s="2"/>
       <c r="AB8" s="2"/>
     </row>
@@ -1233,33 +1365,34 @@
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="4">
-        <v>43689</v>
+        <v>34730</v>
       </c>
       <c r="E9" s="4">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>4632</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="8">
-        <f>SUM(D9:F9)</f>
-        <v>43689</v>
+        <f t="shared" si="1"/>
+        <v>39362</v>
       </c>
       <c r="H9" s="2">
-        <f>10%*G9</f>
-        <v>4368.9000000000005</v>
+        <f t="shared" si="2"/>
+        <v>3936.2000000000003</v>
       </c>
       <c r="I9" s="2">
         <v>400</v>
       </c>
       <c r="J9" s="2">
-        <f>6%*G9</f>
-        <v>2621.3399999999997</v>
+        <f t="shared" si="3"/>
+        <v>2361.7199999999998</v>
       </c>
       <c r="K9" s="8">
-        <f>SUM(G9:J9)</f>
-        <v>51079.24</v>
+        <f t="shared" si="4"/>
+        <v>46059.92</v>
       </c>
       <c r="L9" s="2">
-        <f>2000+3000</f>
+        <f t="shared" si="5"/>
         <v>5000</v>
       </c>
       <c r="M9" s="2">
@@ -1267,47 +1400,47 @@
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="4">
-        <f>SUM(L9:M9)</f>
+        <f t="shared" si="6"/>
         <v>5000</v>
       </c>
       <c r="P9" s="8">
-        <f>K9+O9</f>
-        <v>56079.24</v>
+        <f t="shared" si="7"/>
+        <v>51059.92</v>
       </c>
       <c r="Q9" s="2">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="R9" s="2">
-        <f>H9*2</f>
-        <v>8737.8000000000011</v>
+        <f t="shared" si="8"/>
+        <v>7872.4000000000005</v>
       </c>
       <c r="S9" s="2">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="T9" s="2"/>
       <c r="U9" s="2">
-        <f>J9*2</f>
-        <v>5242.6799999999994</v>
+        <f t="shared" si="9"/>
+        <v>4723.4399999999996</v>
       </c>
       <c r="V9" s="4">
-        <f>SUM(Q9:U9)</f>
-        <v>15781.48</v>
+        <f t="shared" si="10"/>
+        <v>18395.84</v>
       </c>
       <c r="W9" s="2">
-        <f>X9+U9</f>
-        <v>45540.439999999995</v>
+        <f t="shared" si="11"/>
+        <v>37387.519999999997</v>
       </c>
       <c r="X9" s="10">
-        <f>P9-V9</f>
-        <v>40297.759999999995</v>
+        <f t="shared" si="12"/>
+        <v>32664.079999999998</v>
       </c>
       <c r="Y9" s="2">
-        <f>IF(X9*13&gt;600000,1%*X9,0)</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="Z9" s="2">
-        <f>X9-Y9</f>
-        <v>40297.759999999995</v>
+        <f t="shared" si="14"/>
+        <v>32664.079999999998</v>
       </c>
       <c r="AA9" s="2"/>
       <c r="AB9" s="2"/>
@@ -1316,29 +1449,84 @@
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
+      <c r="D10" s="4">
+        <v>34730</v>
+      </c>
+      <c r="E10" s="4">
+        <f t="shared" si="0"/>
+        <v>4632</v>
+      </c>
       <c r="F10" s="2"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
+      <c r="G10" s="8">
+        <f t="shared" si="1"/>
+        <v>39362</v>
+      </c>
+      <c r="H10" s="2">
+        <f t="shared" si="2"/>
+        <v>3936.2000000000003</v>
+      </c>
+      <c r="I10" s="2">
+        <v>400</v>
+      </c>
+      <c r="J10" s="2">
+        <f t="shared" si="3"/>
+        <v>2361.7199999999998</v>
+      </c>
+      <c r="K10" s="8">
+        <f t="shared" si="4"/>
+        <v>46059.92</v>
+      </c>
+      <c r="L10" s="2">
+        <f t="shared" si="5"/>
+        <v>5000</v>
+      </c>
+      <c r="M10" s="2">
+        <v>0</v>
+      </c>
       <c r="N10" s="2"/>
-      <c r="O10" s="4"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
+      <c r="O10" s="4">
+        <f t="shared" si="6"/>
+        <v>5000</v>
+      </c>
+      <c r="P10" s="8">
+        <f t="shared" si="7"/>
+        <v>51059.92</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>800</v>
+      </c>
+      <c r="R10" s="2">
+        <f t="shared" si="8"/>
+        <v>7872.4000000000005</v>
+      </c>
+      <c r="S10" s="2">
+        <v>5000</v>
+      </c>
       <c r="T10" s="2"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="4"/>
-      <c r="W10" s="2"/>
-      <c r="X10" s="10"/>
-      <c r="Y10" s="2"/>
-      <c r="Z10" s="2"/>
+      <c r="U10" s="2">
+        <f t="shared" si="9"/>
+        <v>4723.4399999999996</v>
+      </c>
+      <c r="V10" s="4">
+        <f t="shared" si="10"/>
+        <v>18395.84</v>
+      </c>
+      <c r="W10" s="2">
+        <f t="shared" si="11"/>
+        <v>37387.519999999997</v>
+      </c>
+      <c r="X10" s="10">
+        <f t="shared" si="12"/>
+        <v>32664.079999999998</v>
+      </c>
+      <c r="Y10" s="2">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="Z10" s="2">
+        <f t="shared" si="14"/>
+        <v>32664.079999999998</v>
+      </c>
       <c r="AA10" s="2"/>
       <c r="AB10" s="2"/>
     </row>
@@ -1376,29 +1564,83 @@
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
+      <c r="D12" s="4">
+        <v>43689</v>
+      </c>
+      <c r="E12" s="4">
+        <v>0</v>
+      </c>
       <c r="F12" s="2"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
+      <c r="G12" s="8">
+        <f>SUM(D12:F12)</f>
+        <v>43689</v>
+      </c>
+      <c r="H12" s="2">
+        <f>10%*G12</f>
+        <v>4368.9000000000005</v>
+      </c>
+      <c r="I12" s="2">
+        <v>400</v>
+      </c>
+      <c r="J12" s="2">
+        <f>6%*G12</f>
+        <v>2621.3399999999997</v>
+      </c>
+      <c r="K12" s="8">
+        <f>SUM(G12:J12)</f>
+        <v>51079.24</v>
+      </c>
+      <c r="L12" s="2">
+        <f>2000+3000</f>
+        <v>5000</v>
+      </c>
+      <c r="M12" s="2">
+        <v>0</v>
+      </c>
       <c r="N12" s="2"/>
-      <c r="O12" s="4"/>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
+      <c r="O12" s="4">
+        <f>SUM(L12:M12)</f>
+        <v>5000</v>
+      </c>
+      <c r="P12" s="8">
+        <f>K12+O12</f>
+        <v>56079.24</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>801</v>
+      </c>
+      <c r="R12" s="2">
+        <f>H12*2</f>
+        <v>8737.8000000000011</v>
+      </c>
+      <c r="S12" s="2">
+        <v>1000</v>
+      </c>
       <c r="T12" s="2"/>
-      <c r="U12" s="2"/>
-      <c r="V12" s="4"/>
-      <c r="W12" s="2"/>
-      <c r="X12" s="10"/>
-      <c r="Y12" s="2"/>
-      <c r="Z12" s="2"/>
+      <c r="U12" s="2">
+        <f>J12*2</f>
+        <v>5242.6799999999994</v>
+      </c>
+      <c r="V12" s="4">
+        <f>SUM(Q12:U12)</f>
+        <v>15781.48</v>
+      </c>
+      <c r="W12" s="2">
+        <f>X12+U12</f>
+        <v>45540.439999999995</v>
+      </c>
+      <c r="X12" s="10">
+        <f>P12-V12</f>
+        <v>40297.759999999995</v>
+      </c>
+      <c r="Y12" s="2">
+        <f>IF(X12*13&gt;600000,1%*X12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z12" s="2">
+        <f>X12-Y12</f>
+        <v>40297.759999999995</v>
+      </c>
       <c r="AA12" s="2"/>
       <c r="AB12" s="2"/>
     </row>
@@ -1612,6 +1854,96 @@
       <c r="AA19" s="2"/>
       <c r="AB19" s="2"/>
     </row>
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="8"/>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="2"/>
+      <c r="S20" s="2"/>
+      <c r="T20" s="2"/>
+      <c r="U20" s="2"/>
+      <c r="V20" s="4"/>
+      <c r="W20" s="2"/>
+      <c r="X20" s="10"/>
+      <c r="Y20" s="2"/>
+      <c r="Z20" s="2"/>
+      <c r="AA20" s="2"/>
+      <c r="AB20" s="2"/>
+    </row>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="8"/>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="2"/>
+      <c r="S21" s="2"/>
+      <c r="T21" s="2"/>
+      <c r="U21" s="2"/>
+      <c r="V21" s="4"/>
+      <c r="W21" s="2"/>
+      <c r="X21" s="10"/>
+      <c r="Y21" s="2"/>
+      <c r="Z21" s="2"/>
+      <c r="AA21" s="2"/>
+      <c r="AB21" s="2"/>
+    </row>
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="8"/>
+      <c r="Q22" s="2"/>
+      <c r="R22" s="2"/>
+      <c r="S22" s="2"/>
+      <c r="T22" s="2"/>
+      <c r="U22" s="2"/>
+      <c r="V22" s="4"/>
+      <c r="W22" s="2"/>
+      <c r="X22" s="10"/>
+      <c r="Y22" s="2"/>
+      <c r="Z22" s="2"/>
+      <c r="AA22" s="2"/>
+      <c r="AB22" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="W1:W2"/>

</xml_diff>

<commit_message>
stair and footing left
</commit_message>
<xml_diff>
--- a/New Microsoft Excel Worksheet.xlsx
+++ b/New Microsoft Excel Worksheet.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\082_083\ward1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D8FB979-6E37-4509-AC1A-24150444DD8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,12 +33,13 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>User</author>
+    <author>DELL</author>
   </authors>
   <commentList>
-    <comment ref="D4" authorId="0" shapeId="0" xr:uid="{AD28CD2A-6F95-4BA7-BF55-9966A86999EB}">
+    <comment ref="D4" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -63,7 +63,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{9336CFC1-3459-4BF8-B3A8-5B5478745621}">
+    <comment ref="D5" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -87,7 +87,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{8713AFB4-3DF0-432A-8F9E-0D0B99DA63F9}">
+    <comment ref="D6" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -111,7 +111,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D7" authorId="0" shapeId="0" xr:uid="{B599E665-7579-4A84-B571-B267676937E2}">
+    <comment ref="D7" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -135,7 +135,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D8" authorId="0" shapeId="0" xr:uid="{87073B8F-9072-4EF6-B208-947AACA7D7EC}">
+    <comment ref="D8" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -157,7 +157,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D9" authorId="0" shapeId="0" xr:uid="{5E7E19E1-C15B-4922-ACAF-F55EACE46A00}">
+    <comment ref="D9" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -179,7 +179,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D10" authorId="0" shapeId="0" xr:uid="{DFCBDEA9-2C22-4E5E-9B42-6533BB080AF6}">
+    <comment ref="D10" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -201,7 +201,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D11" authorId="0" shapeId="0" xr:uid="{378A8198-0773-4DBB-81FF-3C343652B837}">
+    <comment ref="D11" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -225,7 +225,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D12" authorId="0" shapeId="0" xr:uid="{A419E87C-F262-442D-8355-622B62EF3E47}">
+    <comment ref="D12" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -249,6 +249,30 @@
         </r>
       </text>
     </comment>
+    <comment ref="D15" authorId="1" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>DELL:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+From shrawan</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -349,7 +373,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -750,31 +774,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AB27"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.140625" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="4.28515625" customWidth="1"/>
-    <col min="4" max="5" width="8.85546875" style="5"/>
-    <col min="6" max="6" width="6.28515625" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" style="9"/>
-    <col min="11" max="11" width="8.85546875" style="9"/>
-    <col min="13" max="13" width="7.28515625" customWidth="1"/>
-    <col min="14" max="14" width="6.42578125" customWidth="1"/>
-    <col min="15" max="15" width="8.5703125" style="5" customWidth="1"/>
+    <col min="1" max="1" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.109375" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="4.33203125" customWidth="1"/>
+    <col min="4" max="5" width="8.88671875" style="5"/>
+    <col min="6" max="6" width="6.33203125" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" style="9"/>
+    <col min="11" max="11" width="8.88671875" style="9"/>
+    <col min="13" max="13" width="7.33203125" customWidth="1"/>
+    <col min="14" max="14" width="6.44140625" customWidth="1"/>
+    <col min="15" max="15" width="8.5546875" style="5" customWidth="1"/>
     <col min="16" max="16" width="8" style="9" customWidth="1"/>
-    <col min="17" max="17" width="6.85546875" customWidth="1"/>
-    <col min="18" max="18" width="7.7109375" customWidth="1"/>
-    <col min="20" max="20" width="8.85546875" customWidth="1"/>
-    <col min="21" max="21" width="14.42578125" customWidth="1"/>
-    <col min="22" max="22" width="8.85546875" style="5"/>
-    <col min="24" max="24" width="8.85546875" style="11"/>
-    <col min="27" max="27" width="8.85546875" customWidth="1"/>
+    <col min="17" max="17" width="6.88671875" customWidth="1"/>
+    <col min="18" max="18" width="7.6640625" customWidth="1"/>
+    <col min="20" max="20" width="8.88671875" customWidth="1"/>
+    <col min="21" max="21" width="14.44140625" customWidth="1"/>
+    <col min="22" max="22" width="8.88671875" style="5"/>
+    <col min="24" max="24" width="8.88671875" style="11"/>
+    <col min="27" max="27" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:28" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -832,7 +856,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="6" customFormat="1" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" s="6" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A2" s="12"/>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -898,7 +922,7 @@
       <c r="AA2" s="12"/>
       <c r="AB2" s="12"/>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -982,7 +1006,7 @@
       <c r="AA3" s="2"/>
       <c r="AB3" s="2"/>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -1068,7 +1092,7 @@
       <c r="AA4" s="2"/>
       <c r="AB4" s="2"/>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -1153,7 +1177,7 @@
       <c r="AA5" s="2"/>
       <c r="AB5" s="2"/>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -1238,7 +1262,7 @@
       <c r="AA6" s="2"/>
       <c r="AB6" s="2"/>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1323,7 +1347,7 @@
       <c r="AA7" s="2"/>
       <c r="AB7" s="2"/>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1355,7 +1379,7 @@
         <v>46059.92</v>
       </c>
       <c r="L8" s="2">
-        <f t="shared" ref="L8:L12" si="5">2000+3000</f>
+        <f t="shared" ref="L8:L15" si="5">2000+3000</f>
         <v>5000</v>
       </c>
       <c r="M8" s="2">
@@ -1408,7 +1432,7 @@
       <c r="AA8" s="2"/>
       <c r="AB8" s="2"/>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1493,7 +1517,7 @@
       <c r="AA9" s="2"/>
       <c r="AB9" s="2"/>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1578,7 +1602,7 @@
       <c r="AA10" s="2"/>
       <c r="AB10" s="2"/>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1665,7 +1689,7 @@
       <c r="AA11" s="2"/>
       <c r="AB11" s="2"/>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -1705,7 +1729,7 @@
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="4">
-        <f t="shared" ref="O11:O12" si="28">SUM(L12:M12)</f>
+        <f t="shared" ref="O12" si="28">SUM(L12:M12)</f>
         <v>5000</v>
       </c>
       <c r="P12" s="8">
@@ -1750,7 +1774,7 @@
       <c r="AA12" s="2"/>
       <c r="AB12" s="2"/>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -1780,121 +1804,123 @@
       <c r="AA13" s="2"/>
       <c r="AB13" s="2"/>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="4">
-        <v>43689</v>
-      </c>
-      <c r="E14" s="4">
-        <v>0</v>
-      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="8">
-        <f>SUM(D14:F14)</f>
-        <v>43689</v>
-      </c>
-      <c r="H14" s="2">
-        <f>10%*G14</f>
-        <v>4368.9000000000005</v>
-      </c>
-      <c r="I14" s="2">
-        <v>400</v>
-      </c>
-      <c r="J14" s="2">
-        <f>6%*G14</f>
-        <v>2621.3399999999997</v>
-      </c>
-      <c r="K14" s="8">
-        <f>SUM(G14:J14)</f>
-        <v>51079.24</v>
-      </c>
-      <c r="L14" s="2">
-        <f>2000+3000</f>
-        <v>5000</v>
-      </c>
-      <c r="M14" s="2">
-        <v>0</v>
-      </c>
+      <c r="G14" s="8"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
       <c r="N14" s="2"/>
-      <c r="O14" s="4">
-        <f>SUM(L14:M14)</f>
-        <v>5000</v>
-      </c>
-      <c r="P14" s="8">
-        <f>K14+O14</f>
-        <v>56079.24</v>
-      </c>
-      <c r="Q14" s="2">
-        <v>801</v>
-      </c>
-      <c r="R14" s="2">
-        <f>H14*2</f>
-        <v>8737.8000000000011</v>
-      </c>
-      <c r="S14" s="2">
-        <v>1000</v>
-      </c>
+      <c r="O14" s="4"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
+      <c r="S14" s="2"/>
       <c r="T14" s="2"/>
-      <c r="U14" s="2">
-        <f>J14*2</f>
-        <v>5242.6799999999994</v>
-      </c>
-      <c r="V14" s="4">
-        <f>SUM(Q14:U14)</f>
-        <v>15781.48</v>
-      </c>
-      <c r="W14" s="2">
-        <f>X14+U14</f>
-        <v>45540.439999999995</v>
-      </c>
-      <c r="X14" s="10">
-        <f>P14-V14</f>
-        <v>40297.759999999995</v>
-      </c>
-      <c r="Y14" s="2">
-        <f>IF(X14*13&gt;600000,1%*X14,0)</f>
-        <v>0</v>
-      </c>
-      <c r="Z14" s="2">
-        <f>X14-Y14</f>
-        <v>40297.759999999995</v>
-      </c>
+      <c r="U14" s="2"/>
+      <c r="V14" s="4"/>
+      <c r="W14" s="2"/>
+      <c r="X14" s="10"/>
+      <c r="Y14" s="2"/>
+      <c r="Z14" s="2"/>
       <c r="AA14" s="2"/>
       <c r="AB14" s="2"/>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
+      <c r="D15" s="4">
+        <f>34730*1.1</f>
+        <v>38203</v>
+      </c>
+      <c r="E15" s="4">
+        <f t="shared" ref="E15" si="29">ROUNDUP(D15/30,0)*4</f>
+        <v>5096</v>
+      </c>
       <c r="F15" s="2"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
+      <c r="G15" s="8">
+        <f t="shared" ref="G15" si="30">SUM(D15:F15)</f>
+        <v>43299</v>
+      </c>
+      <c r="H15" s="2">
+        <f t="shared" ref="H15" si="31">10%*G15</f>
+        <v>4329.9000000000005</v>
+      </c>
+      <c r="I15" s="2">
+        <v>400</v>
+      </c>
+      <c r="J15" s="2">
+        <f t="shared" ref="J15" si="32">6%*G15</f>
+        <v>2597.94</v>
+      </c>
+      <c r="K15" s="8">
+        <f t="shared" ref="K15" si="33">SUM(G15:J15)</f>
+        <v>50626.840000000004</v>
+      </c>
+      <c r="L15" s="2">
+        <f t="shared" si="5"/>
+        <v>5000</v>
+      </c>
+      <c r="M15" s="2">
+        <v>0</v>
+      </c>
       <c r="N15" s="2"/>
-      <c r="O15" s="4"/>
-      <c r="P15" s="8"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
+      <c r="O15" s="4">
+        <f t="shared" ref="O15" si="34">SUM(L15:M15)</f>
+        <v>5000</v>
+      </c>
+      <c r="P15" s="8">
+        <f t="shared" ref="P15" si="35">K15+O15</f>
+        <v>55626.840000000004</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>800</v>
+      </c>
+      <c r="R15" s="2">
+        <f t="shared" ref="R15" si="36">H15*2</f>
+        <v>8659.8000000000011</v>
+      </c>
+      <c r="S15" s="2">
+        <v>5000</v>
+      </c>
       <c r="T15" s="2"/>
-      <c r="U15" s="2"/>
-      <c r="V15" s="4"/>
-      <c r="W15" s="2"/>
-      <c r="X15" s="10"/>
-      <c r="Y15" s="2"/>
-      <c r="Z15" s="2"/>
+      <c r="U15" s="2">
+        <f t="shared" ref="U15" si="37">J15*2</f>
+        <v>5195.88</v>
+      </c>
+      <c r="V15" s="4">
+        <f t="shared" ref="V15" si="38">SUM(Q15:U15)</f>
+        <v>19655.68</v>
+      </c>
+      <c r="W15" s="2">
+        <f t="shared" ref="W15" si="39">X15+U15</f>
+        <v>41167.040000000001</v>
+      </c>
+      <c r="X15" s="10">
+        <f t="shared" ref="X15" si="40">P15-V15</f>
+        <v>35971.160000000003</v>
+      </c>
+      <c r="Y15" s="2">
+        <f t="shared" ref="Y15" si="41">IF(X15*13&gt;600000,1%*X15,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z15" s="2">
+        <f t="shared" ref="Z15" si="42">X15-Y15</f>
+        <v>35971.160000000003</v>
+      </c>
       <c r="AA15" s="2"/>
       <c r="AB15" s="2"/>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -1924,37 +1950,91 @@
       <c r="AA16" s="2"/>
       <c r="AB16" s="2"/>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
+      <c r="D17" s="4">
+        <v>43689</v>
+      </c>
+      <c r="E17" s="4">
+        <v>0</v>
+      </c>
       <c r="F17" s="2"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
+      <c r="G17" s="8">
+        <f>SUM(D17:F17)</f>
+        <v>43689</v>
+      </c>
+      <c r="H17" s="2">
+        <f>10%*G17</f>
+        <v>4368.9000000000005</v>
+      </c>
+      <c r="I17" s="2">
+        <v>400</v>
+      </c>
+      <c r="J17" s="2">
+        <f>6%*G17</f>
+        <v>2621.3399999999997</v>
+      </c>
+      <c r="K17" s="8">
+        <f>SUM(G17:J17)</f>
+        <v>51079.24</v>
+      </c>
+      <c r="L17" s="2">
+        <f>2000+3000</f>
+        <v>5000</v>
+      </c>
+      <c r="M17" s="2">
+        <v>0</v>
+      </c>
       <c r="N17" s="2"/>
-      <c r="O17" s="4"/>
-      <c r="P17" s="8"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="2"/>
+      <c r="O17" s="4">
+        <f>SUM(L17:M17)</f>
+        <v>5000</v>
+      </c>
+      <c r="P17" s="8">
+        <f>K17+O17</f>
+        <v>56079.24</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>801</v>
+      </c>
+      <c r="R17" s="2">
+        <f>H17*2</f>
+        <v>8737.8000000000011</v>
+      </c>
+      <c r="S17" s="2">
+        <v>1000</v>
+      </c>
       <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
-      <c r="V17" s="4"/>
-      <c r="W17" s="2"/>
-      <c r="X17" s="10"/>
-      <c r="Y17" s="2"/>
-      <c r="Z17" s="2"/>
+      <c r="U17" s="2">
+        <f>J17*2</f>
+        <v>5242.6799999999994</v>
+      </c>
+      <c r="V17" s="4">
+        <f>SUM(Q17:U17)</f>
+        <v>15781.48</v>
+      </c>
+      <c r="W17" s="2">
+        <f>X17+U17</f>
+        <v>45540.439999999995</v>
+      </c>
+      <c r="X17" s="10">
+        <f>P17-V17</f>
+        <v>40297.759999999995</v>
+      </c>
+      <c r="Y17" s="2">
+        <f>IF(X17*13&gt;600000,1%*X17,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z17" s="2">
+        <f>X17-Y17</f>
+        <v>40297.759999999995</v>
+      </c>
       <c r="AA17" s="2"/>
       <c r="AB17" s="2"/>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -1984,7 +2064,7 @@
       <c r="AA18" s="2"/>
       <c r="AB18" s="2"/>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -2014,7 +2094,7 @@
       <c r="AA19" s="2"/>
       <c r="AB19" s="2"/>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -2044,7 +2124,7 @@
       <c r="AA20" s="2"/>
       <c r="AB20" s="2"/>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -2074,7 +2154,7 @@
       <c r="AA21" s="2"/>
       <c r="AB21" s="2"/>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -2104,7 +2184,7 @@
       <c r="AA22" s="2"/>
       <c r="AB22" s="2"/>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -2134,7 +2214,7 @@
       <c r="AA23" s="2"/>
       <c r="AB23" s="2"/>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -2164,6 +2244,96 @@
       <c r="AA24" s="2"/>
       <c r="AB24" s="2"/>
     </row>
+    <row r="25" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="2"/>
+      <c r="R25" s="2"/>
+      <c r="S25" s="2"/>
+      <c r="T25" s="2"/>
+      <c r="U25" s="2"/>
+      <c r="V25" s="4"/>
+      <c r="W25" s="2"/>
+      <c r="X25" s="10"/>
+      <c r="Y25" s="2"/>
+      <c r="Z25" s="2"/>
+      <c r="AA25" s="2"/>
+      <c r="AB25" s="2"/>
+    </row>
+    <row r="26" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
+      <c r="N26" s="2"/>
+      <c r="O26" s="4"/>
+      <c r="P26" s="8"/>
+      <c r="Q26" s="2"/>
+      <c r="R26" s="2"/>
+      <c r="S26" s="2"/>
+      <c r="T26" s="2"/>
+      <c r="U26" s="2"/>
+      <c r="V26" s="4"/>
+      <c r="W26" s="2"/>
+      <c r="X26" s="10"/>
+      <c r="Y26" s="2"/>
+      <c r="Z26" s="2"/>
+      <c r="AA26" s="2"/>
+      <c r="AB26" s="2"/>
+    </row>
+    <row r="27" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="2"/>
+      <c r="M27" s="2"/>
+      <c r="N27" s="2"/>
+      <c r="O27" s="4"/>
+      <c r="P27" s="8"/>
+      <c r="Q27" s="2"/>
+      <c r="R27" s="2"/>
+      <c r="S27" s="2"/>
+      <c r="T27" s="2"/>
+      <c r="U27" s="2"/>
+      <c r="V27" s="4"/>
+      <c r="W27" s="2"/>
+      <c r="X27" s="10"/>
+      <c r="Y27" s="2"/>
+      <c r="Z27" s="2"/>
+      <c r="AA27" s="2"/>
+      <c r="AB27" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="W1:W2"/>

</xml_diff>